<commit_message>
Capstone part 2: follow the task order, fuller persona and journey map
The deck and workbook now follow the tasks as set: 1 persona, 2 journey
map, 3 the 5 most important needs, 4 four segments, 5 segment scores,
6 target segment, with numbered section labels, a contents slide and
numbered sheets. The persona gains a "what makes Tunde buy" slide
(triggers, objections, how Tunde chooses and pays); the journey map is
now a single visual map with stage arrows, rows for actions, touchpoints
and thoughts, and a feeling curve, followed by the pain points and
opportunities.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WToQxHdrdWhM7bKqXvUa59
</commit_message>
<xml_diff>
--- a/capstone/Customer_Analysis.xlsx
+++ b/capstone/Customer_Analysis.xlsx
@@ -7,12 +7,12 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="World Data" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Customer Needs" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Segments" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Segment Scores" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Persona" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Journey Map" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1 Persona" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2 Journey Map" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3 Customer Needs" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4 Segments" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5-6 Segment Scores" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="World Data" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
@@ -150,19 +150,47 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="3" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -179,34 +207,6 @@
     </xf>
     <xf numFmtId="9" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
@@ -288,6 +288,181 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr sz="1300" b="0">
+                <a:solidFill>
+                  <a:srgbClr val="404040"/>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr sz="1300" b="0">
+                <a:solidFill>
+                  <a:srgbClr val="404040"/>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+              </a:rPr>
+              <a:t>How Tunde Feels at Each Stage</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+      <overlay val="0"/>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="31750">
+              <a:solidFill>
+                <a:srgbClr val="F2A900"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="circle"/>
+            <size val="9"/>
+            <spPr>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:srgbClr val="202124"/>
+              </a:solidFill>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:solidFill>
+                  <a:srgbClr val="202124"/>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'2 Journey Map'!$B$4:$F$4</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'2 Journey Map'!$B$10:$F$10</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <dLbls>
+          <txPr>
+            <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+            <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:pPr>
+                <a:defRPr sz="1000" b="1">
+                  <a:solidFill>
+                    <a:srgbClr val="262626"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:r>
+                <a:t/>
+              </a:r>
+              <a:endParaRPr sz="1000" b="1">
+                <a:solidFill>
+                  <a:srgbClr val="262626"/>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+              </a:endParaRPr>
+            </a:p>
+          </txPr>
+          <dLblPos val="t"/>
+          <showLegendKey val="0"/>
+          <showVal val="1"/>
+          <showCatName val="0"/>
+          <showSerName val="0"/>
+          <showPercent val="0"/>
+        </dLbls>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <spPr>
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
+            <a:solidFill>
+              <a:srgbClr val="D9D9D9"/>
+            </a:solidFill>
+            <a:prstDash val="solid"/>
+          </a:ln>
+        </spPr>
+        <txPr>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr sz="1000" b="0">
+                <a:solidFill>
+                  <a:srgbClr val="404040"/>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:t/>
+            </a:r>
+            <a:endParaRPr sz="1000" b="0">
+              <a:solidFill>
+                <a:srgbClr val="404040"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+            </a:endParaRPr>
+          </a:p>
+        </txPr>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+          <max val="5"/>
+          <min val="0"/>
+        </scaling>
+        <delete val="1"/>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+        <majorUnit val="1"/>
+      </valAx>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+  <spPr>
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
+      <a:solidFill>
+        <a:srgbClr val="D9D9D9"/>
+      </a:solidFill>
+      <a:prstDash val="solid"/>
+    </a:ln>
+  </spPr>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
@@ -395,12 +570,12 @@
           </dPt>
           <cat>
             <numRef>
-              <f>'Customer Needs'!$A$35:$A$46</f>
+              <f>'3 Customer Needs'!$A$35:$A$46</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Customer Needs'!$B$35:$B$46</f>
+              <f>'3 Customer Needs'!$B$35:$B$46</f>
             </numRef>
           </val>
         </ser>
@@ -509,7 +684,7 @@
 </chartSpace>
 </file>
 
-<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
@@ -569,12 +744,12 @@
           </dPt>
           <cat>
             <numRef>
-              <f>'Segment Scores'!$A$6:$A$9</f>
+              <f>'5-6 Segment Scores'!$A$6:$A$9</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Segment Scores'!$F$6:$F$9</f>
+              <f>'5-6 Segment Scores'!$F$6:$F$9</f>
             </numRef>
           </val>
         </ser>
@@ -683,182 +858,34 @@
 </chartSpace>
 </file>
 
-<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <chart>
-    <title>
-      <tx>
-        <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-            <a:pPr>
-              <a:defRPr sz="1300" b="0">
-                <a:solidFill>
-                  <a:srgbClr val="404040"/>
-                </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:r>
-              <a:rPr sz="1300" b="0">
-                <a:solidFill>
-                  <a:srgbClr val="404040"/>
-                </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
-              </a:rPr>
-              <a:t>How Tunde Feels at Each Stage</a:t>
-            </a:r>
-          </a:p>
-        </rich>
-      </tx>
-      <overlay val="0"/>
-    </title>
-    <plotArea>
-      <lineChart>
-        <grouping val="standard"/>
-        <ser>
-          <idx val="0"/>
-          <order val="0"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="31750">
-              <a:solidFill>
-                <a:srgbClr val="F2A900"/>
-              </a:solidFill>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="circle"/>
-            <size val="9"/>
-            <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:srgbClr val="202124"/>
-              </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:solidFill>
-                  <a:srgbClr val="202124"/>
-                </a:solidFill>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'Journey Map'!$B$4:$F$4</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Journey Map'!$B$10:$F$10</f>
-            </numRef>
-          </val>
-          <smooth val="0"/>
-        </ser>
-        <dLbls>
-          <txPr>
-            <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-            <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:pPr>
-                <a:defRPr sz="1000" b="1">
-                  <a:solidFill>
-                    <a:srgbClr val="262626"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                </a:defRPr>
-              </a:pPr>
-              <a:r>
-                <a:t/>
-              </a:r>
-              <a:endParaRPr sz="1000" b="1">
-                <a:solidFill>
-                  <a:srgbClr val="262626"/>
-                </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
-              </a:endParaRPr>
-            </a:p>
-          </txPr>
-          <dLblPos val="t"/>
-          <showLegendKey val="0"/>
-          <showVal val="1"/>
-          <showCatName val="0"/>
-          <showSerName val="0"/>
-          <showPercent val="0"/>
-        </dLbls>
-        <axId val="10"/>
-        <axId val="100"/>
-      </lineChart>
-      <catAx>
-        <axId val="10"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <delete val="0"/>
-        <axPos val="l"/>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
-            <a:solidFill>
-              <a:srgbClr val="D9D9D9"/>
-            </a:solidFill>
-            <a:prstDash val="solid"/>
-          </a:ln>
-        </spPr>
-        <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-            <a:pPr>
-              <a:defRPr sz="1000" b="0">
-                <a:solidFill>
-                  <a:srgbClr val="404040"/>
-                </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:r>
-              <a:t/>
-            </a:r>
-            <a:endParaRPr sz="1000" b="0">
-              <a:solidFill>
-                <a:srgbClr val="404040"/>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-            </a:endParaRPr>
-          </a:p>
-        </txPr>
-        <crossAx val="100"/>
-        <lblOffset val="100"/>
-      </catAx>
-      <valAx>
-        <axId val="100"/>
-        <scaling>
-          <orientation val="minMax"/>
-          <max val="5"/>
-          <min val="0"/>
-        </scaling>
-        <delete val="1"/>
-        <axPos val="l"/>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="10"/>
-        <majorUnit val="1"/>
-      </valAx>
-    </plotArea>
-    <plotVisOnly val="1"/>
-    <dispBlanksAs val="gap"/>
-  </chart>
-  <spPr>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
-      <a:solidFill>
-        <a:srgbClr val="D9D9D9"/>
-      </a:solidFill>
-      <a:prstDash val="solid"/>
-    </a:ln>
-  </spPr>
-</chartSpace>
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>13</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="7920000" cy="2520000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
@@ -885,7 +912,7 @@
 </wsDr>
 </file>
 
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
@@ -895,33 +922,6 @@
       <rowOff>0</rowOff>
     </from>
     <ext cx="5760000" cy="2340000"/>
-    <graphicFrame>
-      <nvGraphicFramePr>
-        <cNvPr id="1" name="Chart 1"/>
-        <cNvGraphicFramePr/>
-      </nvGraphicFramePr>
-      <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-        </a:graphicData>
-      </a:graphic>
-    </graphicFrame>
-    <clientData/>
-  </oneCellAnchor>
-</wsDr>
-</file>
-
-<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <oneCellAnchor>
-    <from>
-      <col>0</col>
-      <colOff>0</colOff>
-      <row>13</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="7920000" cy="2520000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -1146,375 +1146,699 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D25"/>
+  <dimension ref="A1:B51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="46" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="46" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="70" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1" ht="21" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>CAPSTONE PART 2: CUSTOMER ANALYSIS FOR CYBERSTART</t>
+          <t>1. CUSTOMER PERSONA: TUNDE BAKARE</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>World and Nigerian data behind the customer needs and segments. Found on 11 October 2026.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="22" customHeight="1">
+          <t>A fictional customer from the target segment (Career Switchers), built from the research.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Fact</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>Figure</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>Where</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>Source</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>Fastest-growing skills in the world, 2025 to 2030</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>Networks and cybersecurity: 2nd (after AI and big data)</t>
-        </is>
-      </c>
-      <c r="C5" s="6" t="inlineStr">
-        <is>
-          <t>World</t>
-        </is>
-      </c>
-      <c r="D5" s="5" t="inlineStr">
-        <is>
-          <t>World Economic Forum, Future of Jobs Report 2025 (as summarised by Mwanaspoti)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>Cybersecurity teams with at least one skills gap</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>95%</t>
-        </is>
-      </c>
-      <c r="C6" s="6" t="inlineStr">
-        <is>
-          <t>World</t>
-        </is>
-      </c>
-      <c r="D6" s="5" t="inlineStr">
-        <is>
-          <t>ISC2</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>Skills most in demand in cybersecurity</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>AI and cloud security</t>
-        </is>
-      </c>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
-          <t>World</t>
-        </is>
-      </c>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>ISC2</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>Women in cybersecurity teams</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>22% (26% of professionals under 30)</t>
-        </is>
-      </c>
-      <c r="C8" s="6" t="inlineStr">
-        <is>
-          <t>World</t>
-        </is>
-      </c>
-      <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>ISC2</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>Median age</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>About 19 years</t>
-        </is>
-      </c>
-      <c r="C9" s="6" t="inlineStr">
-        <is>
-          <t>Nigeria</t>
-        </is>
-      </c>
-      <c r="D9" s="5" t="inlineStr">
-        <is>
-          <t>GeoRank, using UN and World Bank data</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>University students</t>
+          <t>Age</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Lives in</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Ikeja, Lagos</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Customer service officer at a phone retailer</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>HND in Business Administration</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Money</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Steady pay above the minimum wage; can spare about ₦50,000 a month</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Devices</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Smartphone and a budget laptop</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>In their words</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>2.1 million</t>
-        </is>
-      </c>
-      <c r="C10" s="6" t="inlineStr">
-        <is>
-          <t>Nigeria</t>
-        </is>
-      </c>
-      <c r="D10" s="5" t="inlineStr">
-        <is>
-          <t>TheCable, reporting the NUC</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>National minimum wage</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>₦70,000 a month</t>
-        </is>
-      </c>
-      <c r="C11" s="6" t="inlineStr">
-        <is>
-          <t>Nigeria</t>
-        </is>
-      </c>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
-          <t>Playroll</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="30" customHeight="1">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>Junior security analyst pay</t>
-        </is>
-      </c>
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t>About ₦150,000 to ₦300,000 a month</t>
-        </is>
-      </c>
-      <c r="C12" s="6" t="inlineStr">
-        <is>
-          <t>Nigeria</t>
-        </is>
-      </c>
-      <c r="D12" s="5" t="inlineStr">
-        <is>
-          <t>Mobility.com.ng</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="30" customHeight="1">
+          <t>“I don't mind paying, if I'm sure it will get me a job.”</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>Goals</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>People using the internet</t>
-        </is>
-      </c>
-      <c r="B13" s="5" t="inlineStr">
-        <is>
-          <t>109 million (end of 2025)</t>
-        </is>
-      </c>
-      <c r="C13" s="6" t="inlineStr">
-        <is>
-          <t>Nigeria</t>
-        </is>
-      </c>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>DataReportal</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="7" t="inlineStr">
-        <is>
-          <t>What the price means for customers (change the yellow cells)</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="22" customHeight="1">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t>Item</t>
-        </is>
-      </c>
-      <c r="B16" s="3" t="inlineStr">
-        <is>
-          <t>Figure</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="5" t="inlineStr">
-        <is>
-          <t>Course price (₦)</t>
-        </is>
-      </c>
-      <c r="B17" s="8" t="n">
-        <v>150000</v>
+          <t>Move into a cybersecurity job within a year</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Earn more: junior analysts earn ₦150,000+ a month</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Learn a skill that will not go out of date</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="n"/>
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>Frustrations</t>
+        </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="5" t="inlineStr">
-        <is>
-          <t>Number of instalments</t>
-        </is>
-      </c>
-      <c r="B18" s="9" t="n">
-        <v>3</v>
-      </c>
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Does not know where to start</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="5" t="inlineStr">
-        <is>
-          <t>National minimum wage a month (₦)</t>
-        </is>
-      </c>
-      <c r="B19" s="8" t="n">
-        <v>70000</v>
-      </c>
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Afraid of paying for a scam course</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="5" t="inlineStr">
-        <is>
-          <t>Junior analyst pay a month, low end (₦)</t>
-        </is>
-      </c>
-      <c r="B20" s="8" t="n">
-        <v>150000</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="4" t="inlineStr">
-        <is>
-          <t>Each instalment (₦)</t>
-        </is>
-      </c>
-      <c r="B21" s="10">
-        <f>B17/B18</f>
-        <v>50000</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="4" t="inlineStr">
-        <is>
-          <t>Months of minimum wage to pay for the course</t>
-        </is>
-      </c>
-      <c r="B22" s="11">
-        <f>ROUND(B17/B19,1)</f>
-        <v>2.1</v>
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Works 8 to 5; free programmes are full</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="n"/>
+    </row>
+    <row r="22" ht="20" customHeight="1">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t>Needs</t>
+        </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>One instalment as a share of the minimum wage</t>
-        </is>
-      </c>
-      <c r="B23" s="12">
-        <f>B17/B18/B19</f>
-        <v>0.714285714285714</v>
-      </c>
+          <t>Hands-on labs at weekends</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>Months of junior analyst pay to earn the price back</t>
-        </is>
-      </c>
-      <c r="B24" s="11">
-        <f>ROUND(B17/B20,1)</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="25" ht="32" customHeight="1">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>So the course is out of reach on the minimum wage, but a junior analyst job earns the price back in about a month: the buyers are people with some income who want a better-paid job.</t>
-        </is>
-      </c>
-      <c r="B25" s="13" t="n"/>
-      <c r="C25" s="13" t="n"/>
-      <c r="D25" s="13" t="n"/>
+          <t>A fair price in 3 parts</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Help when stuck and a route to a job</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="n"/>
+    </row>
+    <row r="27" ht="20" customHeight="1">
+      <c r="A27" s="6" t="inlineStr">
+        <is>
+          <t>Where to reach them</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Google, YouTube and TikTok</t>
+        </is>
+      </c>
+      <c r="B28" s="7" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Facebook groups and WhatsApp</t>
+        </is>
+      </c>
+      <c r="B29" s="7" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>LinkedIn for jobs</t>
+        </is>
+      </c>
+      <c r="B30" s="7" t="n"/>
+    </row>
+    <row r="32" ht="20" customHeight="1">
+      <c r="A32" s="6" t="inlineStr">
+        <is>
+          <t>What makes them buy</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>News of a big data breach, like the CAC breach</t>
+        </is>
+      </c>
+      <c r="B33" s="7" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>A friend who moved into a tech job</t>
+        </is>
+      </c>
+      <c r="B34" s="7" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>A free first class or a deadline to enrol</t>
+        </is>
+      </c>
+      <c r="B35" s="7" t="n"/>
+    </row>
+    <row r="37" ht="20" customHeight="1">
+      <c r="A37" s="6" t="inlineStr">
+        <is>
+          <t>Objections, and our answer</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>“Is it a scam?”  Real reviews and a free first class</t>
+        </is>
+      </c>
+      <c r="B38" s="7" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>“Can I fit it round work?”  Evenings, weekends and recordings</t>
+        </is>
+      </c>
+      <c r="B39" s="7" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>“Will I get a job?”  Exam prep, CV help, employers</t>
+        </is>
+      </c>
+      <c r="B40" s="7" t="n"/>
+    </row>
+    <row r="42" ht="20" customHeight="1">
+      <c r="A42" s="6" t="inlineStr">
+        <is>
+          <t>How they choose</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>Hands-on labs and real tools</t>
+        </is>
+      </c>
+      <c r="B43" s="7" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>The full price and a payment plan</t>
+        </is>
+      </c>
+      <c r="B44" s="7" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>Reviews from past learners</t>
+        </is>
+      </c>
+      <c r="B45" s="7" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>A recognised certificate</t>
+        </is>
+      </c>
+      <c r="B46" s="7" t="n"/>
+    </row>
+    <row r="48" ht="20" customHeight="1">
+      <c r="A48" s="6" t="inlineStr">
+        <is>
+          <t>How they pay</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>₦150,000 in 3 parts of ₦50,000</t>
+        </is>
+      </c>
+      <c r="B49" s="7" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>Pays from salary, a part each month</t>
+        </is>
+      </c>
+      <c r="B50" s="7" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Decides alone; asks friends on WhatsApp first</t>
+        </is>
+      </c>
+      <c r="B51" s="7" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A25:D25"/>
-    <mergeCell ref="A2:D2"/>
-    <mergeCell ref="A15:D15"/>
+  <mergeCells count="35">
+    <mergeCell ref="A48:B48"/>
+    <mergeCell ref="A24:B24"/>
+    <mergeCell ref="A30:B30"/>
+    <mergeCell ref="A15:B15"/>
+    <mergeCell ref="A49:B49"/>
+    <mergeCell ref="A51:B51"/>
+    <mergeCell ref="A45:B45"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A25:B25"/>
+    <mergeCell ref="A37:B37"/>
+    <mergeCell ref="A46:B46"/>
+    <mergeCell ref="A18:B18"/>
+    <mergeCell ref="A27:B27"/>
+    <mergeCell ref="A12:B12"/>
+    <mergeCell ref="A50:B50"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A33:B33"/>
+    <mergeCell ref="A42:B42"/>
+    <mergeCell ref="A32:B32"/>
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="A23:B23"/>
+    <mergeCell ref="A17:B17"/>
+    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="A35:B35"/>
+    <mergeCell ref="A20:B20"/>
+    <mergeCell ref="A38:B38"/>
+    <mergeCell ref="A29:B29"/>
+    <mergeCell ref="A43:B43"/>
+    <mergeCell ref="A19:B19"/>
+    <mergeCell ref="A28:B28"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="A44:B44"/>
+    <mergeCell ref="A40:B40"/>
+    <mergeCell ref="A39:B39"/>
+    <mergeCell ref="A34:B34"/>
   </mergeCells>
   <pageMargins left="0.5" right="0.5" top="0.6" bottom="0.6" header="0.3" footer="0.3"/>
-  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:F12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="21" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>2. CUSTOMER JOURNEY MAP: TUNDE BAKARE</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>From first hearing about cybersecurity to getting a job. Feeling: 1 (very negative) to 5 (very positive).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="24" customHeight="1">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>Stage</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>Awareness</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>Consideration</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>Purchase</t>
+        </is>
+      </c>
+      <c r="E4" s="8" t="inlineStr">
+        <is>
+          <t>Learning</t>
+        </is>
+      </c>
+      <c r="F4" s="8" t="inlineStr">
+        <is>
+          <t>After the course</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="48" customHeight="1">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Doing</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Sees breach news and a TikTok video on cyber careers</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Compares courses, reads reviews, asks in WhatsApp groups</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Joins the free first class, pays the first part</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>Attends classes and weekend labs, takes the exam</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>Applies for jobs, shares the result, refers friends</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="48" customHeight="1">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Touchpoints</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>TikTok, Facebook adverts, Google search</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Website, Google and Trustpilot reviews, WhatsApp</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>Free class, online payment plan</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>Learning platform, Lagos lab, mentor</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>Career help, LinkedIn, alumni group</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="48" customHeight="1">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Thinking and feeling</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>“Can I do this without IT?” Curious but unsure</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>“Is this a scam?” Anxious</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>“I hope it's worth it.” Hopeful, nervous</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>“Hard, but I'm getting it.” Proud</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>“I got the job!” Relieved and proud</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="48" customHeight="1">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Pain points</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>No clear starting point</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Hidden prices, few reviews</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>Big one-off fees</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>Slow support, outdated content</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>No links to employers</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="48" customHeight="1">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Opportunities</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Beginner videos on TikTok and Google</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Publish prices and reviews; fast WhatsApp replies</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>Free first class; 3 instalments</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>Weekly labs, 24-hour support, recordings</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>Exam prep, CV help, employer partners, referral reward</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Feeling (1-5)</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="C10" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D10" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="E10" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="F10" s="9" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Lowest point</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="str">
+        <f>INDEX(B4:F4,MATCH(MIN(B10:F10),B10:F10,0))</f>
+        <v>Consideration</v>
+      </c>
+      <c r="C11" s="7" t="n"/>
+      <c r="D11" s="7" t="n"/>
+      <c r="E11" s="7" t="n"/>
+      <c r="F11" s="7" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Highest point</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="str">
+        <f>INDEX(B4:F4,MATCH(MAX(B10:F10),B10:F10,0))</f>
+        <v>After the course</v>
+      </c>
+      <c r="C12" s="7" t="n"/>
+      <c r="D12" s="7" t="n"/>
+      <c r="E12" s="7" t="n"/>
+      <c r="F12" s="7" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="B12:F12"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="B11:F11"/>
+  </mergeCells>
+  <pageMargins left="0.5" right="0.5" top="0.6" bottom="0.6" header="0.3" footer="0.3"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1536,7 +1860,7 @@
     <row r="1" ht="21" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>CUSTOMER NEEDS: FUNCTIONAL, ECONOMIC, EMOTIONAL AND SOCIAL</t>
+          <t>3. CUSTOMER NEEDS AND THE 5 MOST IMPORTANT</t>
         </is>
       </c>
     </row>
@@ -1548,803 +1872,803 @@
       </c>
     </row>
     <row r="4" ht="32" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="8" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="8" t="inlineStr">
         <is>
           <t>Need</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="8" t="inlineStr">
         <is>
           <t>What it means</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="8" t="inlineStr">
         <is>
           <t>Evidence from the research</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="8" t="inlineStr">
         <is>
           <t>Frequency (1-5)</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" s="8" t="inlineStr">
         <is>
           <t>Impact (1-5)</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" s="8" t="inlineStr">
         <is>
           <t>Importance (of 25)</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="H4" s="8" t="inlineStr">
         <is>
           <t>Rank</t>
         </is>
       </c>
     </row>
     <row r="5" ht="34" customHeight="1">
-      <c r="A5" s="6" t="inlineStr">
+      <c r="A5" s="10" t="inlineStr">
         <is>
           <t>Functional</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>Practical, hands-on skills</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>Labs and real tools, not just theory</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr">
         <is>
           <t>“No labs” and “too much theory” drive low course ratings; TryHackMe is praised for its labs</t>
         </is>
       </c>
-      <c r="E5" s="14" t="n">
+      <c r="E5" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="F5" s="14" t="n">
+      <c r="F5" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="G5" s="15">
+      <c r="G5" s="11">
         <f>E5*F5</f>
         <v>25</v>
       </c>
-      <c r="H5" s="6">
+      <c r="H5" s="10">
         <f>RANK(G5,$G$5:$G$16)</f>
         <v>1</v>
       </c>
     </row>
     <row r="6" ht="34" customHeight="1">
-      <c r="A6" s="6" t="inlineStr">
+      <c r="A6" s="10" t="inlineStr">
         <is>
           <t>Functional</t>
         </is>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>A flexible timetable</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C6" s="4" t="inlineStr">
         <is>
           <t>Evening, weekend and recorded classes</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="D6" s="4" t="inlineStr">
         <is>
           <t>ALX is praised for self-paced study; AltSchool's 20 hours a week was too much for workers</t>
         </is>
       </c>
-      <c r="E6" s="14" t="n">
+      <c r="E6" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="F6" s="14" t="n">
+      <c r="F6" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="G6" s="15">
+      <c r="G6" s="11">
         <f>E6*F6</f>
         <v>16</v>
       </c>
-      <c r="H6" s="6">
+      <c r="H6" s="10">
         <f>RANK(G6,$G$5:$G$16)+COUNTIF($G$5:G5,G6)</f>
         <v>6</v>
       </c>
     </row>
     <row r="7" ht="34" customHeight="1">
-      <c r="A7" s="6" t="inlineStr">
+      <c r="A7" s="10" t="inlineStr">
         <is>
           <t>Functional</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Preparation for a recognised certificate</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr">
+      <c r="C7" s="4" t="inlineStr">
         <is>
           <t>Ready for Security+ or ISC2 CC</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="D7" s="4" t="inlineStr">
         <is>
           <t>Guides say get Security+ first; ISC2's free exam offer ended in May 2026</t>
         </is>
       </c>
-      <c r="E7" s="14" t="n">
+      <c r="E7" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="F7" s="14" t="n">
+      <c r="F7" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="G7" s="15">
+      <c r="G7" s="11">
         <f>E7*F7</f>
         <v>20</v>
       </c>
-      <c r="H7" s="6">
+      <c r="H7" s="10">
         <f>RANK(G7,$G$5:$G$16)+COUNTIF($G$5:G6,G7)</f>
         <v>3</v>
       </c>
     </row>
     <row r="8" ht="34" customHeight="1">
-      <c r="A8" s="6" t="inlineStr">
+      <c r="A8" s="10" t="inlineStr">
         <is>
           <t>Economic</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>An affordable price</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>A fair price for the value</t>
         </is>
       </c>
-      <c r="D8" s="5" t="inlineStr">
+      <c r="D8" s="4" t="inlineStr">
         <is>
           <t>Rising “free course” searches; 20,000+ apply for about 500 free CyberGirls places</t>
         </is>
       </c>
-      <c r="E8" s="14" t="n">
+      <c r="E8" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="F8" s="14" t="n">
+      <c r="F8" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="G8" s="15">
+      <c r="G8" s="11">
         <f>E8*F8</f>
         <v>25</v>
       </c>
-      <c r="H8" s="6">
+      <c r="H8" s="10">
         <f>RANK(G8,$G$5:$G$16)+COUNTIF($G$5:G7,G8)</f>
         <v>2</v>
       </c>
     </row>
     <row r="9" ht="34" customHeight="1">
-      <c r="A9" s="6" t="inlineStr">
+      <c r="A9" s="10" t="inlineStr">
         <is>
           <t>Economic</t>
         </is>
       </c>
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>Paying in instalments</t>
         </is>
       </c>
-      <c r="C9" s="5" t="inlineStr">
+      <c r="C9" s="4" t="inlineStr">
         <is>
           <t>Spread the cost over the course</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr">
+      <c r="D9" s="4" t="inlineStr">
         <is>
           <t>The minimum wage is ₦70,000 a month; a rival lets people pay in parts</t>
         </is>
       </c>
-      <c r="E9" s="14" t="n">
+      <c r="E9" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="F9" s="14" t="n">
+      <c r="F9" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="G9" s="15">
+      <c r="G9" s="11">
         <f>E9*F9</f>
         <v>12</v>
       </c>
-      <c r="H9" s="6">
+      <c r="H9" s="10">
         <f>RANK(G9,$G$5:$G$16)+COUNTIF($G$5:G8,G9)</f>
         <v>8</v>
       </c>
     </row>
     <row r="10" ht="34" customHeight="1">
-      <c r="A10" s="6" t="inlineStr">
+      <c r="A10" s="10" t="inlineStr">
         <is>
           <t>Economic</t>
         </is>
       </c>
-      <c r="B10" s="4" t="inlineStr">
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>A return on the money: a better-paid job</t>
         </is>
       </c>
-      <c r="C10" s="5" t="inlineStr">
+      <c r="C10" s="4" t="inlineStr">
         <is>
           <t>The course pays for itself</t>
         </is>
       </c>
-      <c r="D10" s="5" t="inlineStr">
+      <c r="D10" s="4" t="inlineStr">
         <is>
           <t>Junior analysts earn about ₦150,000 to ₦300,000 a month; people search for salaries</t>
         </is>
       </c>
-      <c r="E10" s="14" t="n">
+      <c r="E10" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="F10" s="14" t="n">
+      <c r="F10" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="G10" s="15">
+      <c r="G10" s="11">
         <f>E10*F10</f>
         <v>20</v>
       </c>
-      <c r="H10" s="6">
+      <c r="H10" s="10">
         <f>RANK(G10,$G$5:$G$16)+COUNTIF($G$5:G9,G10)</f>
         <v>4</v>
       </c>
     </row>
     <row r="11" ht="34" customHeight="1">
-      <c r="A11" s="6" t="inlineStr">
+      <c r="A11" s="10" t="inlineStr">
         <is>
           <t>Emotional</t>
         </is>
       </c>
-      <c r="B11" s="4" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr">
         <is>
           <t>Trust that the course is genuine</t>
         </is>
       </c>
-      <c r="C11" s="5" t="inlineStr">
+      <c r="C11" s="4" t="inlineStr">
         <is>
           <t>Confidence it is not a scam</t>
         </is>
       </c>
-      <c r="D11" s="5" t="inlineStr">
+      <c r="D11" s="4" t="inlineStr">
         <is>
           <t>AltSchool was called a “scam” on X; local providers have few reviews</t>
         </is>
       </c>
-      <c r="E11" s="14" t="n">
+      <c r="E11" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="F11" s="14" t="n">
+      <c r="F11" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="G11" s="15">
+      <c r="G11" s="11">
         <f>E11*F11</f>
         <v>16</v>
       </c>
-      <c r="H11" s="6">
+      <c r="H11" s="10">
         <f>RANK(G11,$G$5:$G$16)+COUNTIF($G$5:G10,G11)</f>
         <v>7</v>
       </c>
     </row>
     <row r="12" ht="34" customHeight="1">
-      <c r="A12" s="6" t="inlineStr">
+      <c r="A12" s="10" t="inlineStr">
         <is>
           <t>Emotional</t>
         </is>
       </c>
-      <c r="B12" s="4" t="inlineStr">
+      <c r="B12" s="3" t="inlineStr">
         <is>
           <t>Feeling supported</t>
         </is>
       </c>
-      <c r="C12" s="5" t="inlineStr">
+      <c r="C12" s="4" t="inlineStr">
         <is>
           <t>Quick help when stuck</t>
         </is>
       </c>
-      <c r="D12" s="5" t="inlineStr">
+      <c r="D12" s="4" t="inlineStr">
         <is>
           <t>Slow support is a complaint about ALX, TryHackMe and AltSchool; 48% of cyber professionals feel exhausted keeping up</t>
         </is>
       </c>
-      <c r="E12" s="14" t="n">
+      <c r="E12" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="F12" s="14" t="n">
+      <c r="F12" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="G12" s="15">
+      <c r="G12" s="11">
         <f>E12*F12</f>
         <v>20</v>
       </c>
-      <c r="H12" s="6">
+      <c r="H12" s="10">
         <f>RANK(G12,$G$5:$G$16)+COUNTIF($G$5:G11,G12)</f>
         <v>5</v>
       </c>
     </row>
     <row r="13" ht="34" customHeight="1">
-      <c r="A13" s="6" t="inlineStr">
+      <c r="A13" s="10" t="inlineStr">
         <is>
           <t>Emotional</t>
         </is>
       </c>
-      <c r="B13" s="4" t="inlineStr">
+      <c r="B13" s="3" t="inlineStr">
         <is>
           <t>Hope for a future-proof career</t>
         </is>
       </c>
-      <c r="C13" s="5" t="inlineStr">
+      <c r="C13" s="4" t="inlineStr">
         <is>
           <t>Pride in a growing field</t>
         </is>
       </c>
-      <c r="D13" s="5" t="inlineStr">
+      <c r="D13" s="4" t="inlineStr">
         <is>
           <t>Cybersecurity is the 2nd fastest-growing skill in the world</t>
         </is>
       </c>
-      <c r="E13" s="14" t="n">
+      <c r="E13" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="F13" s="14" t="n">
+      <c r="F13" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="G13" s="15">
+      <c r="G13" s="11">
         <f>E13*F13</f>
         <v>9</v>
       </c>
-      <c r="H13" s="6">
+      <c r="H13" s="10">
         <f>RANK(G13,$G$5:$G$16)+COUNTIF($G$5:G12,G13)</f>
         <v>9</v>
       </c>
     </row>
     <row r="14" ht="34" customHeight="1">
-      <c r="A14" s="6" t="inlineStr">
+      <c r="A14" s="10" t="inlineStr">
         <is>
           <t>Social</t>
         </is>
       </c>
-      <c r="B14" s="4" t="inlineStr">
+      <c r="B14" s="3" t="inlineStr">
         <is>
           <t>Belonging to a learning community</t>
         </is>
       </c>
-      <c r="C14" s="5" t="inlineStr">
+      <c r="C14" s="4" t="inlineStr">
         <is>
           <t>Learning with others</t>
         </is>
       </c>
-      <c r="D14" s="5" t="inlineStr">
+      <c r="D14" s="4" t="inlineStr">
         <is>
           <t>ALX learners praise its community</t>
         </is>
       </c>
-      <c r="E14" s="14" t="n">
+      <c r="E14" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="F14" s="14" t="n">
+      <c r="F14" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="G14" s="15">
+      <c r="G14" s="11">
         <f>E14*F14</f>
         <v>9</v>
       </c>
-      <c r="H14" s="6">
+      <c r="H14" s="10">
         <f>RANK(G14,$G$5:$G$16)+COUNTIF($G$5:G13,G14)</f>
         <v>10</v>
       </c>
     </row>
     <row r="15" ht="34" customHeight="1">
-      <c r="A15" s="6" t="inlineStr">
+      <c r="A15" s="10" t="inlineStr">
         <is>
           <t>Social</t>
         </is>
       </c>
-      <c r="B15" s="4" t="inlineStr">
+      <c r="B15" s="3" t="inlineStr">
         <is>
           <t>Status of a respected tech job</t>
         </is>
       </c>
-      <c r="C15" s="5" t="inlineStr">
+      <c r="C15" s="4" t="inlineStr">
         <is>
           <t>Being seen as a tech professional</t>
         </is>
       </c>
-      <c r="D15" s="5" t="inlineStr">
+      <c r="D15" s="4" t="inlineStr">
         <is>
           <t>14 million Nigerians are on LinkedIn</t>
         </is>
       </c>
-      <c r="E15" s="14" t="n">
+      <c r="E15" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="F15" s="14" t="n">
+      <c r="F15" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="G15" s="15">
+      <c r="G15" s="11">
         <f>E15*F15</f>
         <v>6</v>
       </c>
-      <c r="H15" s="6">
+      <c r="H15" s="10">
         <f>RANK(G15,$G$5:$G$16)+COUNTIF($G$5:G14,G15)</f>
         <v>12</v>
       </c>
     </row>
     <row r="16" ht="34" customHeight="1">
-      <c r="A16" s="6" t="inlineStr">
+      <c r="A16" s="10" t="inlineStr">
         <is>
           <t>Social</t>
         </is>
       </c>
-      <c r="B16" s="4" t="inlineStr">
+      <c r="B16" s="3" t="inlineStr">
         <is>
           <t>Inclusion for women and non-IT people</t>
         </is>
       </c>
-      <c r="C16" s="5" t="inlineStr">
+      <c r="C16" s="4" t="inlineStr">
         <is>
           <t>Welcome whatever your background</t>
         </is>
       </c>
-      <c r="D16" s="5" t="inlineStr">
+      <c r="D16" s="4" t="inlineStr">
         <is>
           <t>Women are 22% of cyber teams, 26% of those under 30</t>
         </is>
       </c>
-      <c r="E16" s="14" t="n">
+      <c r="E16" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="F16" s="14" t="n">
+      <c r="F16" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="G16" s="15">
+      <c r="G16" s="11">
         <f>E16*F16</f>
         <v>9</v>
       </c>
-      <c r="H16" s="6">
+      <c r="H16" s="10">
         <f>RANK(G16,$G$5:$G$16)+COUNTIF($G$5:G15,G16)</f>
         <v>11</v>
       </c>
     </row>
     <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="7" t="inlineStr">
+      <c r="A18" s="6" t="inlineStr">
         <is>
           <t>The 5 most important needs (found by formula)</t>
         </is>
       </c>
     </row>
     <row r="19" ht="22" customHeight="1">
-      <c r="A19" s="3" t="inlineStr">
+      <c r="A19" s="8" t="inlineStr">
         <is>
           <t>Rank</t>
         </is>
       </c>
-      <c r="B19" s="3" t="inlineStr">
+      <c r="B19" s="8" t="inlineStr">
         <is>
           <t>Need</t>
         </is>
       </c>
-      <c r="C19" s="3" t="inlineStr">
+      <c r="C19" s="8" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="D19" s="3" t="inlineStr">
+      <c r="D19" s="8" t="inlineStr">
         <is>
           <t>Importance (of 25)</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="6" t="n">
+      <c r="A20" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="B20" s="4" t="str">
+      <c r="B20" s="3" t="str">
         <f>INDEX($B$5:$B$16,MATCH(1,$H$5:$H$16,0))</f>
         <v>Practical, hands-on skills</v>
       </c>
-      <c r="C20" s="6" t="str">
+      <c r="C20" s="10" t="str">
         <f>INDEX($A$5:$A$16,MATCH(1,$H$5:$H$16,0))</f>
         <v>Functional</v>
       </c>
-      <c r="D20" s="6">
+      <c r="D20" s="10">
         <f>INDEX($G$5:$G$16,MATCH(1,$H$5:$H$16,0))</f>
         <v>25</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="6" t="n">
+      <c r="A21" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="B21" s="4" t="str">
+      <c r="B21" s="3" t="str">
         <f>INDEX($B$5:$B$16,MATCH(2,$H$5:$H$16,0))</f>
         <v>An affordable price</v>
       </c>
-      <c r="C21" s="6" t="str">
+      <c r="C21" s="10" t="str">
         <f>INDEX($A$5:$A$16,MATCH(2,$H$5:$H$16,0))</f>
         <v>Economic</v>
       </c>
-      <c r="D21" s="6">
+      <c r="D21" s="10">
         <f>INDEX($G$5:$G$16,MATCH(2,$H$5:$H$16,0))</f>
         <v>25</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="6" t="n">
+      <c r="A22" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="B22" s="4" t="str">
+      <c r="B22" s="3" t="str">
         <f>INDEX($B$5:$B$16,MATCH(3,$H$5:$H$16,0))</f>
         <v>Preparation for a recognised certificate</v>
       </c>
-      <c r="C22" s="6" t="str">
+      <c r="C22" s="10" t="str">
         <f>INDEX($A$5:$A$16,MATCH(3,$H$5:$H$16,0))</f>
         <v>Functional</v>
       </c>
-      <c r="D22" s="6">
+      <c r="D22" s="10">
         <f>INDEX($G$5:$G$16,MATCH(3,$H$5:$H$16,0))</f>
         <v>20</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="6" t="n">
+      <c r="A23" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="B23" s="4" t="str">
+      <c r="B23" s="3" t="str">
         <f>INDEX($B$5:$B$16,MATCH(4,$H$5:$H$16,0))</f>
         <v>A return on the money: a better-paid job</v>
       </c>
-      <c r="C23" s="6" t="str">
+      <c r="C23" s="10" t="str">
         <f>INDEX($A$5:$A$16,MATCH(4,$H$5:$H$16,0))</f>
         <v>Economic</v>
       </c>
-      <c r="D23" s="6">
+      <c r="D23" s="10">
         <f>INDEX($G$5:$G$16,MATCH(4,$H$5:$H$16,0))</f>
         <v>20</v>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="6" t="n">
+      <c r="A24" s="10" t="n">
         <v>5</v>
       </c>
-      <c r="B24" s="4" t="str">
+      <c r="B24" s="3" t="str">
         <f>INDEX($B$5:$B$16,MATCH(5,$H$5:$H$16,0))</f>
         <v>Feeling supported</v>
       </c>
-      <c r="C24" s="6" t="str">
+      <c r="C24" s="10" t="str">
         <f>INDEX($A$5:$A$16,MATCH(5,$H$5:$H$16,0))</f>
         <v>Emotional</v>
       </c>
-      <c r="D24" s="6">
+      <c r="D24" s="10">
         <f>INDEX($G$5:$G$16,MATCH(5,$H$5:$H$16,0))</f>
         <v>20</v>
       </c>
     </row>
     <row r="26" ht="20" customHeight="1">
-      <c r="A26" s="7" t="inlineStr">
+      <c r="A26" s="6" t="inlineStr">
         <is>
           <t>Needs by type: average importance</t>
         </is>
       </c>
     </row>
     <row r="27" ht="22" customHeight="1">
-      <c r="A27" s="3" t="inlineStr">
+      <c r="A27" s="8" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="B27" s="3" t="inlineStr">
+      <c r="B27" s="8" t="inlineStr">
         <is>
           <t>Average importance</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="4" t="inlineStr">
+      <c r="A28" s="3" t="inlineStr">
         <is>
           <t>Functional</t>
         </is>
       </c>
-      <c r="B28" s="16">
+      <c r="B28" s="12">
         <f>AVERAGEIF($A$5:$A$16,"Functional",$G$5:$G$16)</f>
         <v>20.3333333333333</v>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="4" t="inlineStr">
+      <c r="A29" s="3" t="inlineStr">
         <is>
           <t>Economic</t>
         </is>
       </c>
-      <c r="B29" s="16">
+      <c r="B29" s="12">
         <f>AVERAGEIF($A$5:$A$16,"Economic",$G$5:$G$16)</f>
         <v>19</v>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="4" t="inlineStr">
+      <c r="A30" s="3" t="inlineStr">
         <is>
           <t>Emotional</t>
         </is>
       </c>
-      <c r="B30" s="16">
+      <c r="B30" s="12">
         <f>AVERAGEIF($A$5:$A$16,"Emotional",$G$5:$G$16)</f>
         <v>15</v>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="4" t="inlineStr">
+      <c r="A31" s="3" t="inlineStr">
         <is>
           <t>Social</t>
         </is>
       </c>
-      <c r="B31" s="16">
+      <c r="B31" s="12">
         <f>AVERAGEIF($A$5:$A$16,"Social",$G$5:$G$16)</f>
         <v>8</v>
       </c>
     </row>
     <row r="33" ht="20" customHeight="1">
-      <c r="A33" s="7" t="inlineStr">
+      <c r="A33" s="6" t="inlineStr">
         <is>
           <t>Importance of each need (chart data)</t>
         </is>
       </c>
     </row>
     <row r="34" ht="22" customHeight="1">
-      <c r="A34" s="3" t="inlineStr">
+      <c r="A34" s="8" t="inlineStr">
         <is>
           <t>Need</t>
         </is>
       </c>
-      <c r="B34" s="3" t="inlineStr">
+      <c r="B34" s="8" t="inlineStr">
         <is>
           <t>Importance</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="5" t="inlineStr">
+      <c r="A35" s="4" t="inlineStr">
         <is>
           <t>Hands-on skills</t>
         </is>
       </c>
-      <c r="B35" s="6">
+      <c r="B35" s="10">
         <f>G5</f>
         <v>25</v>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="5" t="inlineStr">
+      <c r="A36" s="4" t="inlineStr">
         <is>
           <t>Flexible timetable</t>
         </is>
       </c>
-      <c r="B36" s="6">
+      <c r="B36" s="10">
         <f>G6</f>
         <v>16</v>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="5" t="inlineStr">
+      <c r="A37" s="4" t="inlineStr">
         <is>
           <t>Certificate preparation</t>
         </is>
       </c>
-      <c r="B37" s="6">
+      <c r="B37" s="10">
         <f>G7</f>
         <v>20</v>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="5" t="inlineStr">
+      <c r="A38" s="4" t="inlineStr">
         <is>
           <t>Affordable price</t>
         </is>
       </c>
-      <c r="B38" s="6">
+      <c r="B38" s="10">
         <f>G8</f>
         <v>25</v>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="5" t="inlineStr">
+      <c r="A39" s="4" t="inlineStr">
         <is>
           <t>Pay in parts</t>
         </is>
       </c>
-      <c r="B39" s="6">
+      <c r="B39" s="10">
         <f>G9</f>
         <v>12</v>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="5" t="inlineStr">
+      <c r="A40" s="4" t="inlineStr">
         <is>
           <t>Better-paid job</t>
         </is>
       </c>
-      <c r="B40" s="6">
+      <c r="B40" s="10">
         <f>G10</f>
         <v>20</v>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="5" t="inlineStr">
+      <c r="A41" s="4" t="inlineStr">
         <is>
           <t>Trust, not a scam</t>
         </is>
       </c>
-      <c r="B41" s="6">
+      <c r="B41" s="10">
         <f>G11</f>
         <v>16</v>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="5" t="inlineStr">
+      <c r="A42" s="4" t="inlineStr">
         <is>
           <t>Feeling supported</t>
         </is>
       </c>
-      <c r="B42" s="6">
+      <c r="B42" s="10">
         <f>G12</f>
         <v>20</v>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="5" t="inlineStr">
+      <c r="A43" s="4" t="inlineStr">
         <is>
           <t>Future-proof career</t>
         </is>
       </c>
-      <c r="B43" s="6">
+      <c r="B43" s="10">
         <f>G13</f>
         <v>9</v>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="5" t="inlineStr">
+      <c r="A44" s="4" t="inlineStr">
         <is>
           <t>Community</t>
         </is>
       </c>
-      <c r="B44" s="6">
+      <c r="B44" s="10">
         <f>G14</f>
         <v>9</v>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="5" t="inlineStr">
+      <c r="A45" s="4" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="B45" s="6">
+      <c r="B45" s="10">
         <f>G15</f>
         <v>6</v>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="5" t="inlineStr">
+      <c r="A46" s="4" t="inlineStr">
         <is>
           <t>Inclusion</t>
         </is>
       </c>
-      <c r="B46" s="6">
+      <c r="B46" s="10">
         <f>G16</f>
         <v>9</v>
       </c>
@@ -2363,7 +2687,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2382,7 +2706,7 @@
     <row r="1" ht="21" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>FOUR MARKET SEGMENTS</t>
+          <t>4. FOUR MARKET SEGMENTS</t>
         </is>
       </c>
     </row>
@@ -2394,233 +2718,233 @@
       </c>
     </row>
     <row r="4" ht="24" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="8" t="inlineStr">
         <is>
           <t>Base</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="8" t="inlineStr">
         <is>
           <t>Campus Starters</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="8" t="inlineStr">
         <is>
           <t>Career Switchers</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="8" t="inlineStr">
         <is>
           <t>Corporate Upskillers</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="8" t="inlineStr">
         <is>
           <t>Women in Tech Starters</t>
         </is>
       </c>
     </row>
     <row r="5" ht="48" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>Demographic</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>Students and new graduates, 18 to 24; little or no income</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>Working adults, 25 to 35, in non-IT jobs; steady but modest pay</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr">
         <is>
           <t>Staff of banks, telecoms and government, 25 to 45; the employer pays</t>
         </is>
       </c>
-      <c r="E5" s="5" t="inlineStr">
+      <c r="E5" s="4" t="inlineStr">
         <is>
           <t>Women 18 to 30, students and graduates</t>
         </is>
       </c>
     </row>
     <row r="6" ht="48" customHeight="1">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>Geographic</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>University towns across Nigeria; online</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C6" s="4" t="inlineStr">
         <is>
           <t>Lagos, Abuja and Port Harcourt; online in the evenings and at weekends</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="D6" s="4" t="inlineStr">
         <is>
           <t>Head offices in Lagos and Abuja</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr">
+      <c r="E6" s="4" t="inlineStr">
         <is>
           <t>Nationwide, online, with hubs in Lagos and Abuja</t>
         </is>
       </c>
     </row>
     <row r="7" ht="48" customHeight="1">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Psychographic</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>Ambitious and curious; want a head start before graduating</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr">
+      <c r="C7" s="4" t="inlineStr">
         <is>
           <t>Want a better-paid, future-proof career; careful with money</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="D7" s="4" t="inlineStr">
         <is>
           <t>Career growth and doing things by the book</t>
         </is>
       </c>
-      <c r="E7" s="5" t="inlineStr">
+      <c r="E7" s="4" t="inlineStr">
         <is>
           <t>Want a safe, supportive community and role models</t>
         </is>
       </c>
     </row>
     <row r="8" ht="48" customHeight="1">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>Behavioural</t>
         </is>
       </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>Search for “free course”; learn on YouTube and TikTok; very price-driven</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>Compare courses and read reviews; search for salaries; pay in instalments</t>
         </is>
       </c>
-      <c r="D8" s="5" t="inlineStr">
+      <c r="D8" s="4" t="inlineStr">
         <is>
           <t>Buy through HR in groups; want recognised certificates</t>
         </is>
       </c>
-      <c r="E8" s="5" t="inlineStr">
+      <c r="E8" s="4" t="inlineStr">
         <is>
           <t>Apply for free fellowships; follow women's tech groups</t>
         </is>
       </c>
     </row>
     <row r="9" ht="34" customHeight="1">
-      <c r="A9" s="4" t="inlineStr">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>Size evidence</t>
         </is>
       </c>
-      <c r="B9" s="17" t="inlineStr">
+      <c r="B9" s="5" t="inlineStr">
         <is>
           <t>2.1 million university students (NUC)</t>
         </is>
       </c>
-      <c r="C9" s="17" t="inlineStr">
+      <c r="C9" s="5" t="inlineStr">
         <is>
           <t>109 million internet users; median age about 19</t>
         </is>
       </c>
-      <c r="D9" s="17" t="inlineStr">
+      <c r="D9" s="5" t="inlineStr">
         <is>
           <t>Banks, finance and insurance are 29.2% of the cyber market</t>
         </is>
       </c>
-      <c r="E9" s="17" t="inlineStr">
+      <c r="E9" s="5" t="inlineStr">
         <is>
           <t>20,000+ applications a year to CyberGirls</t>
         </is>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="7" t="inlineStr">
+      <c r="A11" s="6" t="inlineStr">
         <is>
           <t>The four bases</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="4" t="inlineStr">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t>Demographic</t>
         </is>
       </c>
-      <c r="B12" s="5" t="inlineStr">
+      <c r="B12" s="4" t="inlineStr">
         <is>
           <t>Age, education, job and income</t>
         </is>
       </c>
-      <c r="C12" s="13" t="n"/>
-      <c r="D12" s="13" t="n"/>
-      <c r="E12" s="13" t="n"/>
+      <c r="C12" s="7" t="n"/>
+      <c r="D12" s="7" t="n"/>
+      <c r="E12" s="7" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="4" t="inlineStr">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>Geographic</t>
         </is>
       </c>
-      <c r="B13" s="5" t="inlineStr">
+      <c r="B13" s="4" t="inlineStr">
         <is>
           <t>Where they live and how they can attend</t>
         </is>
       </c>
-      <c r="C13" s="13" t="n"/>
-      <c r="D13" s="13" t="n"/>
-      <c r="E13" s="13" t="n"/>
+      <c r="C13" s="7" t="n"/>
+      <c r="D13" s="7" t="n"/>
+      <c r="E13" s="7" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="4" t="inlineStr">
+      <c r="A14" s="3" t="inlineStr">
         <is>
           <t>Psychographic</t>
         </is>
       </c>
-      <c r="B14" s="5" t="inlineStr">
+      <c r="B14" s="4" t="inlineStr">
         <is>
           <t>Values, goals, attitudes and lifestyle</t>
         </is>
       </c>
-      <c r="C14" s="13" t="n"/>
-      <c r="D14" s="13" t="n"/>
-      <c r="E14" s="13" t="n"/>
+      <c r="C14" s="7" t="n"/>
+      <c r="D14" s="7" t="n"/>
+      <c r="E14" s="7" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="4" t="inlineStr">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>Behavioural</t>
         </is>
       </c>
-      <c r="B15" s="5" t="inlineStr">
+      <c r="B15" s="4" t="inlineStr">
         <is>
           <t>How they search, decide, buy and learn</t>
         </is>
       </c>
-      <c r="C15" s="13" t="n"/>
-      <c r="D15" s="13" t="n"/>
-      <c r="E15" s="13" t="n"/>
+      <c r="C15" s="7" t="n"/>
+      <c r="D15" s="7" t="n"/>
+      <c r="E15" s="7" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="7">
@@ -2637,7 +2961,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2658,7 +2982,7 @@
     <row r="1" ht="21" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>SEGMENT SCORES</t>
+          <t>5. SEGMENT SCORES AND 6. THE TARGET SEGMENT</t>
         </is>
       </c>
     </row>
@@ -2670,327 +2994,327 @@
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="8" t="inlineStr">
         <is>
           <t>Segment</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="8" t="inlineStr">
         <is>
           <t>Market size</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="8" t="inlineStr">
         <is>
           <t>Accessibility</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="8" t="inlineStr">
         <is>
           <t>Buying potential</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="8" t="inlineStr">
         <is>
           <t>Competition</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" s="8" t="inlineStr">
         <is>
           <t>Weighted score</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" s="8" t="inlineStr">
         <is>
           <t>Rank</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>Weight</t>
         </is>
       </c>
-      <c r="B5" s="18" t="n">
+      <c r="B5" s="13" t="n">
         <v>0.25</v>
       </c>
-      <c r="C5" s="18" t="n">
+      <c r="C5" s="13" t="n">
         <v>0.25</v>
       </c>
-      <c r="D5" s="18" t="n">
+      <c r="D5" s="13" t="n">
         <v>0.3</v>
       </c>
-      <c r="E5" s="18" t="n">
+      <c r="E5" s="13" t="n">
         <v>0.2</v>
       </c>
-      <c r="F5" s="19">
+      <c r="F5" s="14">
         <f>SUM(B5:E5)</f>
         <v>1</v>
       </c>
-      <c r="G5" s="5" t="n"/>
+      <c r="G5" s="4" t="n"/>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>Campus Starters</t>
         </is>
       </c>
-      <c r="B6" s="14" t="n">
+      <c r="B6" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="C6" s="14" t="n">
+      <c r="C6" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="D6" s="14" t="n">
+      <c r="D6" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="E6" s="14" t="n">
+      <c r="E6" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="F6" s="20">
+      <c r="F6" s="15">
         <f>SUMPRODUCT($B$5:$E$5,B6:E6)</f>
         <v>3.25</v>
       </c>
-      <c r="G6" s="6">
+      <c r="G6" s="10">
         <f>RANK(F6,$F$6:$F$9)</f>
         <v>2</v>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Career Switchers</t>
         </is>
       </c>
-      <c r="B7" s="14" t="n">
+      <c r="B7" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="C7" s="14" t="n">
+      <c r="C7" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="D7" s="14" t="n">
+      <c r="D7" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="E7" s="14" t="n">
+      <c r="E7" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="F7" s="20">
+      <c r="F7" s="15">
         <f>SUMPRODUCT($B$5:$E$5,B7:E7)</f>
         <v>4</v>
       </c>
-      <c r="G7" s="6">
+      <c r="G7" s="10">
         <f>RANK(F7,$F$6:$F$9)</f>
         <v>1</v>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>Corporate Upskillers</t>
         </is>
       </c>
-      <c r="B8" s="14" t="n">
+      <c r="B8" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="C8" s="14" t="n">
+      <c r="C8" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="D8" s="14" t="n">
+      <c r="D8" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="E8" s="14" t="n">
+      <c r="E8" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="F8" s="20">
+      <c r="F8" s="15">
         <f>SUMPRODUCT($B$5:$E$5,B8:E8)</f>
         <v>3.15</v>
       </c>
-      <c r="G8" s="6">
+      <c r="G8" s="10">
         <f>RANK(F8,$F$6:$F$9)</f>
         <v>3</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="4" t="inlineStr">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>Women in Tech Starters</t>
         </is>
       </c>
-      <c r="B9" s="14" t="n">
+      <c r="B9" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="C9" s="14" t="n">
+      <c r="C9" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="D9" s="14" t="n">
+      <c r="D9" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="E9" s="14" t="n">
+      <c r="E9" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="F9" s="20">
+      <c r="F9" s="15">
         <f>SUMPRODUCT($B$5:$E$5,B9:E9)</f>
         <v>2.95</v>
       </c>
-      <c r="G9" s="6">
+      <c r="G9" s="10">
         <f>RANK(F9,$F$6:$F$9)</f>
         <v>4</v>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="A11" s="21" t="inlineStr">
-        <is>
-          <t>Target segment</t>
-        </is>
-      </c>
-      <c r="B11" s="22" t="str">
+      <c r="A11" s="16" t="inlineStr">
+        <is>
+          <t>6. Target segment</t>
+        </is>
+      </c>
+      <c r="B11" s="17" t="str">
         <f>INDEX(A6:A9,MATCH(MAX(F6:F9),F6:F9,0))&amp;" ("&amp;TEXT(MAX(F6:F9),"0.00")&amp;" of 5)"</f>
         <v>Career Switchers (4.00 of 5)</v>
       </c>
-      <c r="C11" s="13" t="n"/>
-      <c r="D11" s="13" t="n"/>
-      <c r="E11" s="13" t="n"/>
-      <c r="F11" s="13" t="n"/>
-      <c r="G11" s="13" t="n"/>
+      <c r="C11" s="7" t="n"/>
+      <c r="D11" s="7" t="n"/>
+      <c r="E11" s="7" t="n"/>
+      <c r="F11" s="7" t="n"/>
+      <c r="G11" s="7" t="n"/>
     </row>
     <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="7" t="inlineStr">
+      <c r="A13" s="6" t="inlineStr">
         <is>
           <t>Why each segment got its scores</t>
         </is>
       </c>
     </row>
     <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="3" t="inlineStr">
+      <c r="A14" s="8" t="inlineStr">
         <is>
           <t>Segment</t>
         </is>
       </c>
-      <c r="B14" s="3" t="inlineStr">
+      <c r="B14" s="8" t="inlineStr">
         <is>
           <t>Market size</t>
         </is>
       </c>
-      <c r="C14" s="3" t="inlineStr">
+      <c r="C14" s="8" t="inlineStr">
         <is>
           <t>Accessibility</t>
         </is>
       </c>
-      <c r="D14" s="3" t="inlineStr">
+      <c r="D14" s="8" t="inlineStr">
         <is>
           <t>Buying potential</t>
         </is>
       </c>
-      <c r="E14" s="3" t="inlineStr">
+      <c r="E14" s="8" t="inlineStr">
         <is>
           <t>Competition</t>
         </is>
       </c>
     </row>
     <row r="15" ht="46" customHeight="1">
-      <c r="A15" s="4" t="inlineStr">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>Campus Starters</t>
         </is>
       </c>
-      <c r="B15" s="5" t="inlineStr">
+      <c r="B15" s="4" t="inlineStr">
         <is>
           <t>2.1 million university students</t>
         </is>
       </c>
-      <c r="C15" s="5" t="inlineStr">
+      <c r="C15" s="4" t="inlineStr">
         <is>
           <t>Easy to reach online and on campus</t>
         </is>
       </c>
-      <c r="D15" s="5" t="inlineStr">
+      <c r="D15" s="4" t="inlineStr">
         <is>
           <t>Little income; want free courses</t>
         </is>
       </c>
-      <c r="E15" s="5" t="inlineStr">
+      <c r="E15" s="4" t="inlineStr">
         <is>
           <t>Many free courses aim at them</t>
         </is>
       </c>
     </row>
     <row r="16" ht="46" customHeight="1">
-      <c r="A16" s="4" t="inlineStr">
+      <c r="A16" s="3" t="inlineStr">
         <is>
           <t>Career Switchers</t>
         </is>
       </c>
-      <c r="B16" s="5" t="inlineStr">
+      <c r="B16" s="4" t="inlineStr">
         <is>
           <t>Large: young working adults in big cities</t>
         </is>
       </c>
-      <c r="C16" s="5" t="inlineStr">
+      <c r="C16" s="4" t="inlineStr">
         <is>
           <t>Reach on Facebook, LinkedIn and Google</t>
         </is>
       </c>
-      <c r="D16" s="5" t="inlineStr">
+      <c r="D16" s="4" t="inlineStr">
         <is>
           <t>Earn above the minimum wage; can pay in parts</t>
         </is>
       </c>
-      <c r="E16" s="5" t="inlineStr">
+      <c r="E16" s="4" t="inlineStr">
         <is>
           <t>Few practical, mid-price evening courses</t>
         </is>
       </c>
     </row>
     <row r="17" ht="46" customHeight="1">
-      <c r="A17" s="4" t="inlineStr">
+      <c r="A17" s="3" t="inlineStr">
         <is>
           <t>Corporate Upskillers</t>
         </is>
       </c>
-      <c r="B17" s="5" t="inlineStr">
+      <c r="B17" s="4" t="inlineStr">
         <is>
           <t>Smaller: staff of a few big employers</t>
         </is>
       </c>
-      <c r="C17" s="5" t="inlineStr">
+      <c r="C17" s="4" t="inlineStr">
         <is>
           <t>Slow sales through HR</t>
         </is>
       </c>
-      <c r="D17" s="5" t="inlineStr">
+      <c r="D17" s="4" t="inlineStr">
         <is>
           <t>Employers pay; banks are 29% of the market</t>
         </is>
       </c>
-      <c r="E17" s="5" t="inlineStr">
+      <c r="E17" s="4" t="inlineStr">
         <is>
           <t>Classroom firms already serve them</t>
         </is>
       </c>
     </row>
     <row r="18" ht="46" customHeight="1">
-      <c r="A18" s="4" t="inlineStr">
+      <c r="A18" s="3" t="inlineStr">
         <is>
           <t>Women in Tech Starters</t>
         </is>
       </c>
-      <c r="B18" s="5" t="inlineStr">
+      <c r="B18" s="4" t="inlineStr">
         <is>
           <t>About 1 in 4 cyber professionals under 30</t>
         </is>
       </c>
-      <c r="C18" s="5" t="inlineStr">
+      <c r="C18" s="4" t="inlineStr">
         <is>
           <t>Active online communities</t>
         </is>
       </c>
-      <c r="D18" s="5" t="inlineStr">
+      <c r="D18" s="4" t="inlineStr">
         <is>
           <t>Often students; want free places</t>
         </is>
       </c>
-      <c r="E18" s="5" t="inlineStr">
+      <c r="E18" s="4" t="inlineStr">
         <is>
           <t>Free fellowships, but places are few</t>
         </is>
@@ -3009,552 +3333,377 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="1"/>
-  </sheetPr>
-  <dimension ref="A1:B30"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="70" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="21" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>CUSTOMER PERSONA: TUNDE BAKARE</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>A fictional customer from the target segment (Career Switchers), built from the research.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>Age</t>
-        </is>
-      </c>
-      <c r="B4" s="5" t="inlineStr">
-        <is>
-          <t>27</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>Lives in</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>Ikeja, Lagos</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>Job</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>Customer service officer at a phone retailer</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>Education</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>HND in Business Administration</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>Money</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>Steady pay above the minimum wage; can spare about ₦50,000 a month</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>Devices</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>Smartphone and a budget laptop</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>In their words</t>
-        </is>
-      </c>
-      <c r="B10" s="17" t="inlineStr">
-        <is>
-          <t>“I don't mind paying, if I'm sure it will get me a job.”</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="7" t="inlineStr">
-        <is>
-          <t>Goals</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="5" t="inlineStr">
-        <is>
-          <t>Move into a cybersecurity job within a year</t>
-        </is>
-      </c>
-      <c r="B13" s="13" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="5" t="inlineStr">
-        <is>
-          <t>Earn more: junior analysts earn ₦150,000+ a month</t>
-        </is>
-      </c>
-      <c r="B14" s="13" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="5" t="inlineStr">
-        <is>
-          <t>Learn a skill that will not go out of date</t>
-        </is>
-      </c>
-      <c r="B15" s="13" t="n"/>
-    </row>
-    <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="7" t="inlineStr">
-        <is>
-          <t>Frustrations</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="5" t="inlineStr">
-        <is>
-          <t>Does not know where to start</t>
-        </is>
-      </c>
-      <c r="B18" s="13" t="n"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="5" t="inlineStr">
-        <is>
-          <t>Afraid of paying for a scam course</t>
-        </is>
-      </c>
-      <c r="B19" s="13" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="5" t="inlineStr">
-        <is>
-          <t>Works 8 to 5; free programmes are full</t>
-        </is>
-      </c>
-      <c r="B20" s="13" t="n"/>
-    </row>
-    <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="7" t="inlineStr">
-        <is>
-          <t>Needs</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="5" t="inlineStr">
-        <is>
-          <t>Hands-on labs at weekends</t>
-        </is>
-      </c>
-      <c r="B23" s="13" t="n"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="5" t="inlineStr">
-        <is>
-          <t>A fair price in 3 parts</t>
-        </is>
-      </c>
-      <c r="B24" s="13" t="n"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="5" t="inlineStr">
-        <is>
-          <t>Help when stuck and a route to a job</t>
-        </is>
-      </c>
-      <c r="B25" s="13" t="n"/>
-    </row>
-    <row r="27" ht="20" customHeight="1">
-      <c r="A27" s="7" t="inlineStr">
-        <is>
-          <t>Where to reach them</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="5" t="inlineStr">
-        <is>
-          <t>Google, YouTube and TikTok</t>
-        </is>
-      </c>
-      <c r="B28" s="13" t="n"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="5" t="inlineStr">
-        <is>
-          <t>Facebook groups and WhatsApp</t>
-        </is>
-      </c>
-      <c r="B29" s="13" t="n"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="5" t="inlineStr">
-        <is>
-          <t>LinkedIn for jobs</t>
-        </is>
-      </c>
-      <c r="B30" s="13" t="n"/>
-    </row>
-  </sheetData>
-  <mergeCells count="18">
-    <mergeCell ref="A20:B20"/>
-    <mergeCell ref="A24:B24"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A30:B30"/>
-    <mergeCell ref="A15:B15"/>
-    <mergeCell ref="A29:B29"/>
-    <mergeCell ref="A25:B25"/>
-    <mergeCell ref="A19:B19"/>
-    <mergeCell ref="A23:B23"/>
-    <mergeCell ref="A28:B28"/>
-    <mergeCell ref="A13:B13"/>
-    <mergeCell ref="A14:B14"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="A17:B17"/>
-    <mergeCell ref="A18:B18"/>
-    <mergeCell ref="A27:B27"/>
-    <mergeCell ref="A22:B22"/>
-    <mergeCell ref="A12:B12"/>
-  </mergeCells>
-  <pageMargins left="0.5" right="0.5" top="0.6" bottom="0.6" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1"/>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:D25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
-    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="46" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="46" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1" ht="21" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>CUSTOMER JOURNEY MAP: TUNDE BAKARE</t>
+          <t>CAPSTONE PART 2: CUSTOMER ANALYSIS FOR CYBERSTART</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>From first hearing about cybersecurity to getting a job. Feeling: 1 (very negative) to 5 (very positive).</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="24" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>Stage</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>Awareness</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>Consideration</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>Purchase</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>Learning</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>After the course</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="48" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>Doing</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>Sees breach news and a TikTok video on cyber careers</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
-          <t>Compares courses, reads reviews, asks in WhatsApp groups</t>
-        </is>
-      </c>
-      <c r="D5" s="5" t="inlineStr">
-        <is>
-          <t>Joins the free first class, pays the first part</t>
-        </is>
-      </c>
-      <c r="E5" s="5" t="inlineStr">
-        <is>
-          <t>Attends classes and weekend labs, takes the exam</t>
-        </is>
-      </c>
-      <c r="F5" s="5" t="inlineStr">
-        <is>
-          <t>Applies for jobs, shares the result, refers friends</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="48" customHeight="1">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>Touchpoints</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>TikTok, Facebook adverts, Google search</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>Website, Google and Trustpilot reviews, WhatsApp</t>
-        </is>
-      </c>
-      <c r="D6" s="5" t="inlineStr">
-        <is>
-          <t>Free class, online payment plan</t>
-        </is>
-      </c>
-      <c r="E6" s="5" t="inlineStr">
-        <is>
-          <t>Learning platform, Lagos lab, mentor</t>
-        </is>
-      </c>
-      <c r="F6" s="5" t="inlineStr">
-        <is>
-          <t>Career help, LinkedIn, alumni group</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="48" customHeight="1">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>Thinking and feeling</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>“Can I do this without IT?” Curious but unsure</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>“Is this a scam?” Anxious</t>
-        </is>
-      </c>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>“I hope it's worth it.” Hopeful, nervous</t>
-        </is>
-      </c>
-      <c r="E7" s="5" t="inlineStr">
-        <is>
-          <t>“Hard, but I'm getting it.” Proud</t>
-        </is>
-      </c>
-      <c r="F7" s="5" t="inlineStr">
-        <is>
-          <t>“I got the job!” Relieved and proud</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="48" customHeight="1">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>Pain points</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>No clear starting point</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>Hidden prices, few reviews</t>
-        </is>
-      </c>
-      <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>Big one-off fees</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="inlineStr">
-        <is>
-          <t>Slow support, outdated content</t>
-        </is>
-      </c>
-      <c r="F8" s="5" t="inlineStr">
-        <is>
-          <t>No links to employers</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="48" customHeight="1">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>Opportunities</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>Beginner videos on TikTok and Google</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t>Publish prices and reviews; fast WhatsApp replies</t>
-        </is>
-      </c>
-      <c r="D9" s="5" t="inlineStr">
-        <is>
-          <t>Free first class; 3 instalments</t>
-        </is>
-      </c>
-      <c r="E9" s="5" t="inlineStr">
-        <is>
-          <t>Weekly labs, 24-hour support, recordings</t>
-        </is>
-      </c>
-      <c r="F9" s="5" t="inlineStr">
-        <is>
-          <t>Exam prep, CV help, employer partners, referral reward</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>Feeling (1-5)</t>
-        </is>
-      </c>
-      <c r="B10" s="14" t="n">
+          <t>World and Nigerian data behind the customer needs and segments. Found on 11 October 2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>Fact</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>Figure</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>Where</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Fastest-growing skills in the world, 2025 to 2030</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Networks and cybersecurity: 2nd (after AI and big data)</t>
+        </is>
+      </c>
+      <c r="C5" s="10" t="inlineStr">
+        <is>
+          <t>World</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>World Economic Forum, Future of Jobs Report 2025 (as summarised by Mwanaspoti)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Cybersecurity teams with at least one skills gap</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>95%</t>
+        </is>
+      </c>
+      <c r="C6" s="10" t="inlineStr">
+        <is>
+          <t>World</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>ISC2</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Skills most in demand in cybersecurity</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>AI and cloud security</t>
+        </is>
+      </c>
+      <c r="C7" s="10" t="inlineStr">
+        <is>
+          <t>World</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>ISC2</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Women in cybersecurity teams</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>22% (26% of professionals under 30)</t>
+        </is>
+      </c>
+      <c r="C8" s="10" t="inlineStr">
+        <is>
+          <t>World</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>ISC2</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Median age</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>About 19 years</t>
+        </is>
+      </c>
+      <c r="C9" s="10" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>GeoRank, using UN and World Bank data</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>University students</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>2.1 million</t>
+        </is>
+      </c>
+      <c r="C10" s="10" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>TheCable, reporting the NUC</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>National minimum wage</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>₦70,000 a month</t>
+        </is>
+      </c>
+      <c r="C11" s="10" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>Playroll</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Junior security analyst pay</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>About ₦150,000 to ₦300,000 a month</t>
+        </is>
+      </c>
+      <c r="C12" s="10" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>Mobility.com.ng</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>People using the internet</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>109 million (end of 2025)</t>
+        </is>
+      </c>
+      <c r="C13" s="10" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>DataReportal</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>What the price means for customers (change the yellow cells)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="22" customHeight="1">
+      <c r="A16" s="8" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B16" s="8" t="inlineStr">
+        <is>
+          <t>Figure</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Course price (₦)</t>
+        </is>
+      </c>
+      <c r="B17" s="18" t="n">
+        <v>150000</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Number of instalments</t>
+        </is>
+      </c>
+      <c r="B18" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="C10" s="14" t="n">
-        <v>2</v>
-      </c>
-      <c r="D10" s="14" t="n">
-        <v>3</v>
-      </c>
-      <c r="E10" s="14" t="n">
-        <v>4</v>
-      </c>
-      <c r="F10" s="14" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>Lowest point</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="str">
-        <f>INDEX(B4:F4,MATCH(MIN(B10:F10),B10:F10,0))</f>
-        <v>Consideration</v>
-      </c>
-      <c r="C11" s="13" t="n"/>
-      <c r="D11" s="13" t="n"/>
-      <c r="E11" s="13" t="n"/>
-      <c r="F11" s="13" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>Highest point</t>
-        </is>
-      </c>
-      <c r="B12" s="4" t="str">
-        <f>INDEX(B4:F4,MATCH(MAX(B10:F10),B10:F10,0))</f>
-        <v>After the course</v>
-      </c>
-      <c r="C12" s="13" t="n"/>
-      <c r="D12" s="13" t="n"/>
-      <c r="E12" s="13" t="n"/>
-      <c r="F12" s="13" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>National minimum wage a month (₦)</t>
+        </is>
+      </c>
+      <c r="B19" s="18" t="n">
+        <v>70000</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Junior analyst pay a month, low end (₦)</t>
+        </is>
+      </c>
+      <c r="B20" s="18" t="n">
+        <v>150000</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Each instalment (₦)</t>
+        </is>
+      </c>
+      <c r="B21" s="20">
+        <f>B17/B18</f>
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>Months of minimum wage to pay for the course</t>
+        </is>
+      </c>
+      <c r="B22" s="21">
+        <f>ROUND(B17/B19,1)</f>
+        <v>2.1</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>One instalment as a share of the minimum wage</t>
+        </is>
+      </c>
+      <c r="B23" s="22">
+        <f>B17/B18/B19</f>
+        <v>0.714285714285714</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>Months of junior analyst pay to earn the price back</t>
+        </is>
+      </c>
+      <c r="B24" s="21">
+        <f>ROUND(B17/B20,1)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" ht="32" customHeight="1">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>So the course is out of reach on the minimum wage, but a junior analyst job earns the price back in about a month: the buyers are people with some income who want a better-paid job.</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="n"/>
+      <c r="C25" s="7" t="n"/>
+      <c r="D25" s="7" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="B12:F12"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="B11:F11"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A25:D25"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A15:D15"/>
   </mergeCells>
   <pageMargins left="0.5" right="0.5" top="0.6" bottom="0.6" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -3588,37 +3737,37 @@
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="8" t="inlineStr">
         <is>
           <t>No.</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="8" t="inlineStr">
         <is>
           <t>Who</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="8" t="inlineStr">
         <is>
           <t>What</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="8" t="inlineStr">
         <is>
           <t>Link</t>
         </is>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="6" t="n">
+      <c r="A5" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>World Economic Forum, Future of Jobs Report 2025 (as summarised by Mwanaspoti)</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>Networks and cybersecurity is the second fastest-growing skill, after AI and big data</t>
         </is>
@@ -3630,15 +3779,15 @@
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="6" t="n">
+      <c r="A6" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>ISC2</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C6" s="4" t="inlineStr">
         <is>
           <t>2025 Cybersecurity Workforce Study (16,029 professionals, December 2025)</t>
         </is>
@@ -3650,15 +3799,15 @@
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="6" t="n">
+      <c r="A7" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>ISC2</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr">
+      <c r="C7" s="4" t="inlineStr">
         <is>
           <t>Women comprise 22 percent of the cybersecurity workforce (March 2025)</t>
         </is>
@@ -3670,15 +3819,15 @@
       </c>
     </row>
     <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="6" t="n">
+      <c r="A8" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>TheCable, reporting the NUC</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>NUC: only one percent of Nigerian population in universities</t>
         </is>
@@ -3690,15 +3839,15 @@
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="6" t="n">
+      <c r="A9" s="10" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>Playroll</t>
         </is>
       </c>
-      <c r="C9" s="5" t="inlineStr">
+      <c r="C9" s="4" t="inlineStr">
         <is>
           <t>Minimum wage in Nigeria in 2026 (National Minimum Wage (Amendment) Act 2024)</t>
         </is>
@@ -3710,15 +3859,15 @@
       </c>
     </row>
     <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="6" t="n">
+      <c r="A10" s="10" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="4" t="inlineStr">
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>GeoRank, using UN and World Bank data</t>
         </is>
       </c>
-      <c r="C10" s="5" t="inlineStr">
+      <c r="C10" s="4" t="inlineStr">
         <is>
           <t>Demographics of Nigeria</t>
         </is>
@@ -3730,15 +3879,15 @@
       </c>
     </row>
     <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="6" t="n">
+      <c r="A11" s="10" t="n">
         <v>7</v>
       </c>
-      <c r="B11" s="4" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr">
         <is>
           <t>Google Trends</t>
         </is>
       </c>
-      <c r="C11" s="5" t="inlineStr">
+      <c r="C11" s="4" t="inlineStr">
         <is>
           <t>Market Research Lab Task 1 screenshots, 28 September 2026: Nigeria, past 12 months, all categories, web search</t>
         </is>
@@ -3750,15 +3899,15 @@
       </c>
     </row>
     <row r="12" ht="30" customHeight="1">
-      <c r="A12" s="6" t="n">
+      <c r="A12" s="10" t="n">
         <v>8</v>
       </c>
-      <c r="B12" s="4" t="inlineStr">
+      <c r="B12" s="3" t="inlineStr">
         <is>
           <t>DataReportal</t>
         </is>
       </c>
-      <c r="C12" s="5" t="inlineStr">
+      <c r="C12" s="4" t="inlineStr">
         <is>
           <t>Digital 2026: Nigeria</t>
         </is>
@@ -3770,15 +3919,15 @@
       </c>
     </row>
     <row r="13" ht="30" customHeight="1">
-      <c r="A13" s="6" t="n">
+      <c r="A13" s="10" t="n">
         <v>9</v>
       </c>
-      <c r="B13" s="4" t="inlineStr">
+      <c r="B13" s="3" t="inlineStr">
         <is>
           <t>NapoleonCat</t>
         </is>
       </c>
-      <c r="C13" s="5" t="inlineStr">
+      <c r="C13" s="4" t="inlineStr">
         <is>
           <t>Social media users in Nigeria, 2026 (Facebook, Instagram, LinkedIn)</t>
         </is>
@@ -3790,15 +3939,15 @@
       </c>
     </row>
     <row r="14" ht="30" customHeight="1">
-      <c r="A14" s="6" t="n">
+      <c r="A14" s="10" t="n">
         <v>10</v>
       </c>
-      <c r="B14" s="4" t="inlineStr">
+      <c r="B14" s="3" t="inlineStr">
         <is>
           <t>Mobility.com.ng</t>
         </is>
       </c>
-      <c r="C14" s="5" t="inlineStr">
+      <c r="C14" s="4" t="inlineStr">
         <is>
           <t>Cybersecurity career path: jobs and pay in Nigeria</t>
         </is>
@@ -3810,15 +3959,15 @@
       </c>
     </row>
     <row r="15" ht="30" customHeight="1">
-      <c r="A15" s="6" t="n">
+      <c r="A15" s="10" t="n">
         <v>11</v>
       </c>
-      <c r="B15" s="4" t="inlineStr">
+      <c r="B15" s="3" t="inlineStr">
         <is>
           <t>Mordor Intelligence</t>
         </is>
       </c>
-      <c r="C15" s="5" t="inlineStr">
+      <c r="C15" s="4" t="inlineStr">
         <is>
           <t>Nigeria Cybersecurity Market: size and share</t>
         </is>
@@ -3830,15 +3979,15 @@
       </c>
     </row>
     <row r="16" ht="30" customHeight="1">
-      <c r="A16" s="6" t="n">
+      <c r="A16" s="10" t="n">
         <v>12</v>
       </c>
-      <c r="B16" s="4" t="inlineStr">
+      <c r="B16" s="3" t="inlineStr">
         <is>
           <t>Security Blue Team</t>
         </is>
       </c>
-      <c r="C16" s="5" t="inlineStr">
+      <c r="C16" s="4" t="inlineStr">
         <is>
           <t>CyberGirls Fellowship success stories</t>
         </is>
@@ -3850,15 +3999,15 @@
       </c>
     </row>
     <row r="17" ht="30" customHeight="1">
-      <c r="A17" s="6" t="n">
+      <c r="A17" s="10" t="n">
         <v>13</v>
       </c>
-      <c r="B17" s="4" t="inlineStr">
+      <c r="B17" s="3" t="inlineStr">
         <is>
           <t>TechCabal</t>
         </is>
       </c>
-      <c r="C17" s="5" t="inlineStr">
+      <c r="C17" s="4" t="inlineStr">
         <is>
           <t>AltSchool Africa set out to fix education. Now it's learning its own lessons (29 October 2025)</t>
         </is>
@@ -3870,15 +4019,15 @@
       </c>
     </row>
     <row r="18" ht="30" customHeight="1">
-      <c r="A18" s="6" t="n">
+      <c r="A18" s="10" t="n">
         <v>14</v>
       </c>
-      <c r="B18" s="4" t="inlineStr">
+      <c r="B18" s="3" t="inlineStr">
         <is>
           <t>Techpoint Africa</t>
         </is>
       </c>
-      <c r="C18" s="5" t="inlineStr">
+      <c r="C18" s="4" t="inlineStr">
         <is>
           <t>AltSchool Africa Nano-Diploma</t>
         </is>
@@ -3890,15 +4039,15 @@
       </c>
     </row>
     <row r="19" ht="30" customHeight="1">
-      <c r="A19" s="6" t="n">
+      <c r="A19" s="10" t="n">
         <v>15</v>
       </c>
-      <c r="B19" s="4" t="inlineStr">
+      <c r="B19" s="3" t="inlineStr">
         <is>
           <t>Trustpilot</t>
         </is>
       </c>
-      <c r="C19" s="5" t="inlineStr">
+      <c r="C19" s="4" t="inlineStr">
         <is>
           <t>ALX Africa reviews</t>
         </is>
@@ -3910,15 +4059,15 @@
       </c>
     </row>
     <row r="20" ht="30" customHeight="1">
-      <c r="A20" s="6" t="n">
+      <c r="A20" s="10" t="n">
         <v>16</v>
       </c>
-      <c r="B20" s="4" t="inlineStr">
+      <c r="B20" s="3" t="inlineStr">
         <is>
           <t>Trustpilot</t>
         </is>
       </c>
-      <c r="C20" s="5" t="inlineStr">
+      <c r="C20" s="4" t="inlineStr">
         <is>
           <t>TryHackMe reviews</t>
         </is>
@@ -3930,15 +4079,15 @@
       </c>
     </row>
     <row r="21" ht="30" customHeight="1">
-      <c r="A21" s="6" t="n">
+      <c r="A21" s="10" t="n">
         <v>17</v>
       </c>
-      <c r="B21" s="4" t="inlineStr">
+      <c r="B21" s="3" t="inlineStr">
         <is>
           <t>Course.careers</t>
         </is>
       </c>
-      <c r="C21" s="5" t="inlineStr">
+      <c r="C21" s="4" t="inlineStr">
         <is>
           <t>Overview of course reviews: what drives low ratings</t>
         </is>
@@ -3950,15 +4099,15 @@
       </c>
     </row>
     <row r="22" ht="30" customHeight="1">
-      <c r="A22" s="6" t="n">
+      <c r="A22" s="10" t="n">
         <v>18</v>
       </c>
-      <c r="B22" s="4" t="inlineStr">
+      <c r="B22" s="3" t="inlineStr">
         <is>
           <t>vLearnSecurity</t>
         </is>
       </c>
-      <c r="C22" s="5" t="inlineStr">
+      <c r="C22" s="4" t="inlineStr">
         <is>
           <t>Pricing: 12-week foundational course</t>
         </is>
@@ -3970,15 +4119,15 @@
       </c>
     </row>
     <row r="23" ht="30" customHeight="1">
-      <c r="A23" s="6" t="n">
+      <c r="A23" s="10" t="n">
         <v>19</v>
       </c>
-      <c r="B23" s="4" t="inlineStr">
+      <c r="B23" s="3" t="inlineStr">
         <is>
           <t>ISC2</t>
         </is>
       </c>
-      <c r="C23" s="5" t="inlineStr">
+      <c r="C23" s="4" t="inlineStr">
         <is>
           <t>One Million Certified in Cybersecurity: conclusion (April 2026)</t>
         </is>
@@ -3990,15 +4139,15 @@
       </c>
     </row>
     <row r="24" ht="30" customHeight="1">
-      <c r="A24" s="6" t="n">
+      <c r="A24" s="10" t="n">
         <v>20</v>
       </c>
-      <c r="B24" s="4" t="inlineStr">
+      <c r="B24" s="3" t="inlineStr">
         <is>
           <t>Profolio.ng</t>
         </is>
       </c>
-      <c r="C24" s="5" t="inlineStr">
+      <c r="C24" s="4" t="inlineStr">
         <is>
           <t>How to get a cybersecurity analyst job in Nigeria</t>
         </is>

</xml_diff>